<commit_message>
27th March 2025 Update
</commit_message>
<xml_diff>
--- a/Compititor's_Price/Recticel_Prices/Recticel_Prices_24-03-2025.xlsx
+++ b/Compititor's_Price/Recticel_Prices/Recticel_Prices_24-03-2025.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Priyanka\Documents\Price_Comp_Dashboard\Compititor's_Price\Recticel_Prices\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5738CAEE-CCDB-4A93-AB4D-4AEF341CB9DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3416369B-D6B6-4E46-994F-35926E98D0A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1281,6 +1281,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:S25"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="68.85546875" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">

</xml_diff>